<commit_message>
P/N list: add full Sage article references
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/PN_Perenco_26-57-CM.xlsx
+++ b/PN_Perenco_26-57-CM.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,8 +50,11 @@
     <font>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Consolas"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +69,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2A8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7A8"/>
       </patternFill>
     </fill>
   </fills>
@@ -95,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -119,6 +127,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -516,7 +530,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Jaune = à compléter avant envoi (référence fabricant, fiche technique). Les P/N ENEDRIL sont une proposition à valider.</t>
+          <t>Jaune = à compléter avant envoi. Orange = à vérifier (2 articles avec la même référence Sage). Les P/N ENEDRIL sont une proposition à valider.</t>
         </is>
       </c>
     </row>
@@ -553,7 +567,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Réf. fabricant (Ref.)</t>
+          <t>Réf. article Sage (Ref.)</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -594,7 +608,11 @@
           <t>ENE-931XIN-01</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr"/>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>931XINSXOVX5838</t>
+        </is>
+      </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -629,7 +647,11 @@
           <t>ENE-931XIN-02</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr"/>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>931XINSXSEMOVX5838</t>
+        </is>
+      </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -664,7 +686,11 @@
           <t>ENE-931XM-01</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr"/>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>931XMUSTINSXSQ38</t>
+        </is>
+      </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -699,7 +725,11 @@
           <t>ENE-932XB-01</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr"/>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>932XBRAZFLUX</t>
+        </is>
+      </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -734,7 +764,11 @@
           <t>ENE-932XB-02</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr"/>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>932XBRAZBZ5</t>
+        </is>
+      </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -769,7 +803,11 @@
           <t>ENE-932XB-03</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr"/>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>932XBRAZFLUX</t>
+        </is>
+      </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -804,7 +842,11 @@
           <t>ENE-932XB-04</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr"/>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>932XBRAZAG</t>
+        </is>
+      </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -839,7 +881,11 @@
           <t>ENE-930XM-01</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr"/>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>930XMUSTLOY14</t>
+        </is>
+      </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -874,7 +920,11 @@
           <t>ENE-930XM-02</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr"/>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>930XMUSTLOYY18</t>
+        </is>
+      </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -909,7 +959,11 @@
           <t>ENE-930XM-03</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr"/>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>930XMUSTLOY316</t>
+        </is>
+      </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -944,7 +998,11 @@
           <t>ENE-936XM-01</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr"/>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>936XMASQUEPROTEC</t>
+        </is>
+      </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -979,7 +1037,11 @@
           <t>ENE-936XC-01</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr"/>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>936XCAGOULEINTE</t>
+        </is>
+      </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -1014,7 +1076,11 @@
           <t>ENE-936XC-02</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr"/>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>936XCOUVERTUREDET</t>
+        </is>
+      </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -1049,7 +1115,11 @@
           <t>ENE-936XT-01</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr"/>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>936XTABLIERALUMINE</t>
+        </is>
+      </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -1084,7 +1154,11 @@
           <t>ENE-935XT-01</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr"/>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>935XTORCHWELD</t>
+        </is>
+      </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -1119,7 +1193,11 @@
           <t>ENE-935XD-01</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr"/>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>935XDETENOXY</t>
+        </is>
+      </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -1154,7 +1232,11 @@
           <t>ENE-935XD-02</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr"/>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>935XDETENACETY</t>
+        </is>
+      </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -1189,7 +1271,11 @@
           <t>ENE-935XT-02</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr"/>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>935XTUYAUOXAD</t>
+        </is>
+      </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -1224,7 +1310,11 @@
           <t>ENE-935XA-01</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr"/>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>935XANTIRETOURACET</t>
+        </is>
+      </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -1259,7 +1349,11 @@
           <t>ENE-935XA-02</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr"/>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>935XANTIRETOUROXY</t>
+        </is>
+      </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -1294,7 +1388,11 @@
           <t>ENE-935XR-01</t>
         </is>
       </c>
-      <c r="G26" s="7" t="inlineStr"/>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>935XRACCORDFEM</t>
+        </is>
+      </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -1329,7 +1427,11 @@
           <t>ENE-935XR-02</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr"/>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>935XRACCORDFEMAC</t>
+        </is>
+      </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -1364,7 +1466,11 @@
           <t>ENE-935XE-01</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr"/>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>935XEMBOUTMALE</t>
+        </is>
+      </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -1399,7 +1505,11 @@
           <t>ENE-935XT-03</t>
         </is>
       </c>
-      <c r="G29" s="7" t="inlineStr"/>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>935XTHERMODIGI</t>
+        </is>
+      </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
           <t>À joindre</t>
@@ -1434,9 +1544,9 @@
           <t>ENE-901XP-01</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>N/A (service)</t>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>à compléter (ligne non visible)</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">

</xml_diff>

<commit_message>
P/N list: use full Sage reference as stable P/N
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/PN_Perenco_26-57-CM.xlsx
+++ b/PN_Perenco_26-57-CM.xlsx
@@ -103,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -132,6 +132,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -530,7 +533,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Jaune = à compléter avant envoi. Orange = à vérifier (2 articles avec la même référence Sage). Les P/N ENEDRIL sont une proposition à valider.</t>
+          <t>Le P/N ENEDRIL est la référence article Sage complète : il est identique dans tous les devis. Jaune = à compléter. Orange = à vérifier (même référence pour 2 articles).</t>
         </is>
       </c>
     </row>
@@ -562,7 +565,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>P/N ENEDRIL (proposé)</t>
+          <t>P/N ENEDRIL</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -605,7 +608,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>ENE-931XIN-01</t>
+          <t>931XINSXOVX5838</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
@@ -644,7 +647,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>ENE-931XIN-02</t>
+          <t>931XINSXSEMOVX5838</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -683,7 +686,7 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>ENE-931XM-01</t>
+          <t>931XMUSTINSXSQ38</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -722,7 +725,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>ENE-932XB-01</t>
+          <t>932XBRAZFLUX</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr">
@@ -761,7 +764,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>ENE-932XB-02</t>
+          <t>932XBRAZBZ5</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -800,7 +803,7 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>ENE-932XB-03</t>
+          <t>932XBRAZFLUX</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -839,7 +842,7 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>ENE-932XB-04</t>
+          <t>932XBRAZAG</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
@@ -878,7 +881,7 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>ENE-930XM-01</t>
+          <t>930XMUSTLOY14</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -917,7 +920,7 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>ENE-930XM-02</t>
+          <t>930XMUSTLOYY18</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
@@ -956,7 +959,7 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>ENE-930XM-03</t>
+          <t>930XMUSTLOY316</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
@@ -995,7 +998,7 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>ENE-936XM-01</t>
+          <t>936XMASQUEPROTEC</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -1034,7 +1037,7 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>ENE-936XC-01</t>
+          <t>936XCAGOULEINTE</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
@@ -1073,7 +1076,7 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>ENE-936XC-02</t>
+          <t>936XCOUVERTUREDET</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
@@ -1112,7 +1115,7 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>ENE-936XT-01</t>
+          <t>936XTABLIERALUMINE</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
@@ -1151,7 +1154,7 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>ENE-935XT-01</t>
+          <t>935XTORCHWELD</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
@@ -1190,7 +1193,7 @@
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>ENE-935XD-01</t>
+          <t>935XDETENOXY</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
@@ -1229,7 +1232,7 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>ENE-935XD-02</t>
+          <t>935XDETENACETY</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
@@ -1268,7 +1271,7 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>ENE-935XT-02</t>
+          <t>935XTUYAUOXAD</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
@@ -1307,7 +1310,7 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>ENE-935XA-01</t>
+          <t>935XANTIRETOURACET</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
@@ -1346,7 +1349,7 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>ENE-935XA-02</t>
+          <t>935XANTIRETOUROXY</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
@@ -1385,7 +1388,7 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>ENE-935XR-01</t>
+          <t>935XRACCORDFEM</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
@@ -1424,7 +1427,7 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>ENE-935XR-02</t>
+          <t>935XRACCORDFEMAC</t>
         </is>
       </c>
       <c r="G27" s="10" t="inlineStr">
@@ -1463,7 +1466,7 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>ENE-935XE-01</t>
+          <t>935XEMBOUTMALE</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
@@ -1502,7 +1505,7 @@
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>ENE-935XT-03</t>
+          <t>935XTHERMODIGI</t>
         </is>
       </c>
       <c r="G29" s="10" t="inlineStr">
@@ -1539,9 +1542,9 @@
           <t>Unit</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>ENE-901XP-01</t>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>à compléter</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -1576,51 +1579,43 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>Règle de codification des P/N ENEDRIL (proposition)</t>
+          <t>Règle de P/N ENEDRIL</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Format : ENE-&lt;code article Sage&gt;-&lt;NN&gt;</t>
+          <t>P/N = référence article Sage complète (ex. 931XINSXOVX5838).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>&lt;code article Sage&gt; : code déjà présent sur le devis (ex. 931XIN, 935XT).</t>
+          <t>Elle est liée à l'article, pas au devis : le même article porte toujours le même P/N, quel que soit l'ordre des lignes ou le client.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>&lt;NN&gt; : numéro d'ordre à 2 chiffres au sein du même code article, dans l'ordre du devis.</t>
+          <t>Un article distinct (taille, matière, conditionnement) a sa propre référence Sage, donc son propre P/N.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Exemple : les 3 articles du code 935XT deviennent ENE-935XT-01, -02 et -03.</t>
+          <t>Le code à 6 caractères imprimé sur le devis (ex. 931XIN) est un code famille : il ne doit pas servir de P/N.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Un P/N = un article distinct : taille, matière ou conditionnement différents donnent un P/N différent.</t>
-        </is>
-      </c>
+      <c r="A6" s="9" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>La colonne « Réf. fabricant » reste à renseigner avec les références du catalogue du fabricant ou du fournisseur : elles ne peuvent pas être déduites du devis.</t>
-        </is>
-      </c>
+      <c r="A7" s="9" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
P/N list: descriptive product-based P/N distinct from Sage ref
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPwnZBmWUGhvYebrP3X3Z2
</commit_message>
<xml_diff>
--- a/PN_Perenco_26-57-CM.xlsx
+++ b/PN_Perenco_26-57-CM.xlsx
@@ -533,7 +533,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Le P/N ENEDRIL est la référence article Sage complète : il est identique dans tous les devis. Jaune = à compléter. Orange = à vérifier (même référence pour 2 articles).</t>
+          <t>Ref. = référence article Sage. P/N = code produit ENEDRIL, identique dans tous les devis (proposition à valider). Jaune = à compléter. Orange = à vérifier.</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>P/N ENEDRIL</t>
+          <t>P/N ENEDRIL (proposé)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>931XINSXOVX5838</t>
+          <t>ENE-INS-OV-58-38-14</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>931XINSXSEMOVX5838</t>
+          <t>ENE-INS-SOV-516-38-14</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -686,7 +686,7 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>931XMUSTINSXSQ38</t>
+          <t>ENE-INS-SQ-38-38-14</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>932XBRAZFLUX</t>
+          <t>ENE-BRZ-FLUX808-CU-200G</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>932XBRAZBZ5</t>
+          <t>ENE-BRZ-50BZ-5KG</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>932XBRAZFLUX</t>
+          <t>ENE-BRZ-FLUX808-AG-200G</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>932XBRAZAG</t>
+          <t>ENE-BRZ-50AG-1KG</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>930XMUSTLOY14</t>
+          <t>ENE-LOY-14-10LB</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>930XMUSTLOYY18</t>
+          <t>ENE-LOY-18-10LB</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>930XMUSTLOY316</t>
+          <t>ENE-LOY-316-10LB</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>936XMASQUEPROTEC</t>
+          <t>ENE-EPI-MASQUE-ENGLOB</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>936XCAGOULEINTE</t>
+          <t>ENE-EPI-CAGOULE-VENT</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>936XCOUVERTUREDET</t>
+          <t>ENE-EPI-COUV-900</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>936XTABLIERALUMINE</t>
+          <t>ENE-EPI-TABLIER-ALU</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>935XTORCHWELD</t>
+          <t>ENE-OXY-CHALUMEAU</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>935XDETENOXY</t>
+          <t>ENE-OXY-DETEND-OX</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>935XDETENACETY</t>
+          <t>ENE-OXY-DETEND-AC</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>935XTUYAUOXAD</t>
+          <t>ENE-OXY-TUYAU-OXAD</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>935XANTIRETOURACET</t>
+          <t>ENE-OXY-ANTIRET-AC</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>935XANTIRETOUROXY</t>
+          <t>ENE-OXY-ANTIRET-OX</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>935XRACCORDFEM</t>
+          <t>ENE-OXY-RACC-F-OX</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>935XRACCORDFEMAC</t>
+          <t>ENE-OXY-RACC-F-AC</t>
         </is>
       </c>
       <c r="G27" s="10" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>935XEMBOUTMALE</t>
+          <t>ENE-OXY-EMBOUT-M</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>935XTHERMODIGI</t>
+          <t>ENE-THERMO-IR</t>
         </is>
       </c>
       <c r="G29" s="10" t="inlineStr">
@@ -1542,9 +1542,9 @@
           <t>Unit</t>
         </is>
       </c>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>à compléter</t>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>ENE-SRV-PACK</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -1579,40 +1579,44 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>Règle de P/N ENEDRIL</t>
+          <t>Règle de P/N ENEDRIL (proposition)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>P/N = référence article Sage complète (ex. 931XINSXOVX5838).</t>
+          <t>Format : ENE-&lt;famille&gt;-&lt;caractéristiques du produit&gt;, sans numéro d'ordre.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Elle est liée à l'article, pas au devis : le même article porte toujours le même P/N, quel que soit l'ordre des lignes ou le client.</t>
+          <t>Familles : INS inserts · BRZ brasure et flux · LOY baguettes · EPI équipements de protection · OXY matériel oxy-acétylène · THERMO mesure · SRV services.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>Un article distinct (taille, matière, conditionnement) a sa propre référence Sage, donc son propre P/N.</t>
+          <t>Les chiffres sont les dimensions ou le conditionnement du produit (ex. INS-OV-58-38-14 = insert ovale 5/8 x 3/8 x 1/4 ; LOY-18-10LB = baguettes 1/8 en boîte de 10 lbs).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Le code à 6 caractères imprimé sur le devis (ex. 931XIN) est un code famille : il ne doit pas servir de P/N.</t>
+          <t>Le P/N décrit le produit, pas la ligne du devis : le même article a le même P/N quels que soient le devis, le client ou l'ordre des lignes.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="n"/>
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Ref. = référence article Sage complète. P/N et Ref. sont donc deux codes différents.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n"/>

</xml_diff>